<commit_message>
feat: centralize organization and custodian unit name to Virtual Nursing Simulation Learning Center
</commit_message>
<xml_diff>
--- a/reports_sample/รายงานทะเบียนพัสดุและครุภัณฑ์รวม_ตัวอย่าง.xlsx
+++ b/reports_sample/รายงานทะเบียนพัสดุและครุภัณฑ์รวม_ตัวอย่าง.xlsx
@@ -422,7 +422,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ส่วนราชการ: คณะพยาบาลศาสตร์       หน่วยงานผู้ครอบครอง: ศูนย์ฝึกทักษะการพยาบาล (Nursing Lab)       ประเภท: ครุภัณฑ์การแพทย์และฝึกทักษะ</v>
+        <v>ส่วนราชการ: คณะพยาบาลศาสตร์ มหาวิทยาลัยเกษตรศาสตร์       หน่วยงานผู้ครอบครอง: ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง       ประเภท: ครุภัณฑ์การแพทย์และฝึกทักษะ</v>
       </c>
     </row>
     <row r="3">
@@ -506,7 +506,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L6" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M6" t="str">
         <v>-</v>
@@ -547,7 +547,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L7" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M7" t="str">
         <v>-</v>
@@ -588,7 +588,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L8" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M8" t="str">
         <v>-</v>
@@ -629,7 +629,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L9" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M9" t="str">
         <v>-</v>
@@ -670,7 +670,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L10" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M10" t="str">
         <v>-</v>
@@ -711,7 +711,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L11" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M11" t="str">
         <v>-</v>
@@ -752,7 +752,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L12" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M12" t="str">
         <v>-</v>
@@ -793,7 +793,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L13" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M13" t="str">
         <v>-</v>
@@ -834,7 +834,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L14" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M14" t="str">
         <v>-</v>
@@ -875,7 +875,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L15" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M15" t="str">
         <v>-</v>
@@ -916,7 +916,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L16" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M16" t="str">
         <v>-</v>
@@ -957,7 +957,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L17" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M17" t="str">
         <v>-</v>
@@ -998,7 +998,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L18" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M18" t="str">
         <v>-</v>
@@ -1039,7 +1039,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L19" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M19" t="str">
         <v>-</v>
@@ -1080,7 +1080,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L20" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M20" t="str">
         <v>-</v>
@@ -1121,7 +1121,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L21" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M21" t="str">
         <v>-</v>
@@ -1162,7 +1162,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L22" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M22" t="str">
         <v>-</v>
@@ -1203,7 +1203,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L23" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M23" t="str">
         <v>-</v>
@@ -1244,7 +1244,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L24" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M24" t="str">
         <v>-</v>
@@ -1285,7 +1285,7 @@
         <v>พร้อมใช้งาน</v>
       </c>
       <c r="L25" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล คณะพยาบาลศาสตร์</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง คณะพยาบาลศาสตร์</v>
       </c>
       <c r="M25" t="str">
         <v>-</v>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ส่วนราชการ: คณะพยาบาลศาสตร์       หน่วยงานผู้ครอบครอง: ศูนย์ฝึกทักษะการพยาบาล (Nursing Lab)       ประเภท: วัสดุการแพทย์และเวชภัณฑ์สิ้นเปลือง</v>
+        <v>ส่วนราชการ: คณะพยาบาลศาสตร์ มหาวิทยาลัยเกษตรศาสตร์       หน่วยงานผู้ครอบครอง: ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง       ประเภท: วัสดุการแพทย์และเวชภัณฑ์สิ้นเปลือง</v>
       </c>
     </row>
     <row r="3">
@@ -1723,7 +1723,7 @@
         <v>เซต</v>
       </c>
       <c r="F9" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G9" t="str">
         <v>9999</v>
@@ -1805,7 +1805,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F11" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G11" t="str">
         <v>9999</v>
@@ -1846,7 +1846,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F12" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G12" t="str">
         <v>9999</v>
@@ -1887,7 +1887,7 @@
         <v>ขวด</v>
       </c>
       <c r="F13" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G13" t="str">
         <v>อว 6501.38/1429</v>
@@ -1928,7 +1928,7 @@
         <v>ขวด</v>
       </c>
       <c r="F14" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G14" t="str">
         <v>อว 6501.38/1106</v>
@@ -1969,7 +1969,7 @@
         <v>ขวด</v>
       </c>
       <c r="F15" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G15" t="str">
         <v>อว 6501.38/1429</v>
@@ -2010,7 +2010,7 @@
         <v>ขวด</v>
       </c>
       <c r="F16" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G16" t="str">
         <v>อว 6501.38/1106</v>
@@ -2051,7 +2051,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F17" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G17" t="str">
         <v>9999</v>
@@ -2092,7 +2092,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F18" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G18" t="str">
         <v>9999</v>
@@ -2133,7 +2133,7 @@
         <v>ขวด</v>
       </c>
       <c r="F19" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G19" t="str">
         <v>9999</v>
@@ -2174,7 +2174,7 @@
         <v>แพ๊ค</v>
       </c>
       <c r="F20" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G20" t="str">
         <v>111</v>
@@ -2215,7 +2215,7 @@
         <v>แพ๊ค</v>
       </c>
       <c r="F21" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G21" t="str">
         <v>1414</v>
@@ -2256,7 +2256,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F22" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G22" t="str">
         <v>อว 6501.38/1429</v>
@@ -2297,7 +2297,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F23" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G23" t="str">
         <v>อว 6501.38/1429</v>
@@ -2338,7 +2338,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F24" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G24" t="str">
         <v>9999</v>
@@ -2379,7 +2379,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F25" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G25" t="str">
         <v>อว 6501.38/1429</v>
@@ -2420,7 +2420,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F26" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G26" t="str">
         <v>9999</v>
@@ -2461,7 +2461,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F27" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G27" t="str">
         <v>9999</v>
@@ -2502,7 +2502,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F28" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G28" t="str">
         <v>อว 6501.38/1429</v>
@@ -2543,7 +2543,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F29" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G29" t="str">
         <v>9999</v>
@@ -2584,7 +2584,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F30" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G30" t="str">
         <v>อว 6501.38/1429</v>
@@ -2625,7 +2625,7 @@
         <v>กล่อง</v>
       </c>
       <c r="F31" t="str">
-        <v>ศูนย์ฝึกทักษะการพยาบาล</v>
+        <v>ศูนย์การเรียนรู้ปฏิบัติการทางการพยาบาลเสมือนจริง</v>
       </c>
       <c r="G31" t="str">
         <v>อว 6501.38/1429</v>

</xml_diff>